<commit_message>
Add Arabic (RTL) language toggle for Maaden client
EN/AR language switcher in the sidebar (cookie-backed, POST /api/v1/locale).
Arabic sets lang=ar + dir=rtl on <html>; RTL CSS flips tree indentation and
right-aligns table headers while keeping tag IDs / codes LTR.

Light i18n layer: client-safe dictionary (src/lib/i18n-dict.ts) + server
helper tServer() (src/lib/i18n.ts). Translated chrome, nav, screen titles,
crumbs, KPI labels, section headers, lifecycle chips, compliance families,
common buttons and table headers. Domain data (tags, standards codes,
property names) stays language-neutral by design.

Verified in browser: AR renders dir=rtl with Arabic nav/KPIs/registry
headers + lifecycle chips; toggling back returns lang=en/ltr. Demo arc
unaffected (data untranslated). DB reset to pristine seed.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/RFQ Doc/2026.07.06 Maaden SoW - Clarifications + XDH Assumptions v2.xlsx
+++ b/RFQ Doc/2026.07.06 Maaden SoW - Clarifications + XDH Assumptions v2.xlsx
@@ -521,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" style="1" min="1" max="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Quesries</t>
+          <t>Queries</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>12 months Year 1 implementation following the SoW 3.3.10 phase structure</t>
+          <t>10 months (40 weeks) Year 1 implementation per XDH Master Roadmap XDH-AE-Q26-05-00030, following the SoW 3.3.10 phase structure</t>
         </is>
       </c>
     </row>
@@ -611,7 +611,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Phase 4 = Weeks 17 to 52 (8 months) ending at Go-Live and Final Acceptance</t>
+          <t>Phase 4 = Weeks 17 to 40, split 4a-4d (M1 CDE W17-24, M4 Quality W21-29, M5 Procurement W25-32, Handover W33-40), ending at Final Acceptance W40</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Year 1: M1+M2+M3 pilot then production from W17, M4 Phase 1 baseline, M5 baseline only. Year 2: M2/M3 full production, M4 Phase 2, M5 production</t>
+          <t>Single 40-week programme per Master Roadmap: Phase 2 pilots M2 AWP + M3 Pre-Comm (W5-12); Phase 4 delivers M1 CDE, M4 Quality, M5 Procurement to full production; all 5 modules live by W40. Years 2-5 = maintenance + enhancements</t>
         </is>
       </c>
     </row>

</xml_diff>